<commit_message>
Polish submission ownership wording
</commit_message>
<xml_diff>
--- a/data/federer_companies_pune.xlsx
+++ b/data/federer_companies_pune.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Federer Pipeline" sheetId="1" r:id="R877af5c8ccc04f1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Log" sheetId="2" r:id="Rb2ce04b334fa43d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="Ra60b2e539bc44056"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Federer Pipeline" sheetId="1" r:id="R89c163feabdc4cb0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Log" sheetId="2" r:id="R3625d2d29f4d47db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R3cd32ac68149488d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2390,7 +2390,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
-        <x:v>Prepared for</x:v>
+        <x:v>Submitted by</x:v>
       </x:c>
       <x:c r="B12" t="str">
         <x:v>Souradeep Ghosh</x:v>

</xml_diff>